<commit_message>
data(queue): Casual 최대 대기 30초 -> 10초
필요 인원이 최대 대기에 걸쳐 정원->최소로 선형 감소한다(spec 6-2 정정).
정원 8/최소 2면 10초에 걸쳐 8->2로 줄고, 사람이 모이면 그 전에 출발한다.
지금까지는 대기 시간이 코드에 5로 하드코딩돼 이 값이 쓰이지 않았다.
</commit_message>
<xml_diff>
--- a/table/Datas/#Queue.xlsx
+++ b/table/Datas/#Queue.xlsx
@@ -546,21 +546,11 @@
           <t>##group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -666,7 +656,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat(masterdata): TbQueue에 ticket_ttl_seconds 추가 (그룹 m)
대기표 절대 상한. 매칭서버만 읽으므로 그룹 m으로 좁혀 클라 빌드에 안 싣는다.
시작값은 두 큐 모두 600초(10분) — Open Match assignedDeleteTimeout과 같은 눈금.
</commit_message>
<xml_diff>
--- a/table/Datas/#Queue.xlsx
+++ b/table/Datas/#Queue.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,11 @@
           <t>max_wait_seconds</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ticket_ttl_seconds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,6 +544,11 @@
           <t>int</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -551,6 +561,11 @@
           <t>c</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -611,6 +626,11 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>max_wait_seconds</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>ticket_ttl_seconds</t>
         </is>
       </c>
     </row>
@@ -658,6 +678,9 @@
       <c r="L5" t="n">
         <v>10</v>
       </c>
+      <c r="M5" t="n">
+        <v>600</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="n">
@@ -702,6 +725,9 @@
       </c>
       <c r="L6" t="n">
         <v>60</v>
+      </c>
+      <c r="M6" t="n">
+        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>